<commit_message>
fix: gate private CSV pilot delivery on data quality and review
</commit_message>
<xml_diff>
--- a/docs/weekly_report.xlsx
+++ b/docs/weekly_report.xlsx
@@ -515,29 +515,65 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>【美澜风尚旗舰店】电商经营分析周报</t>
+          <t>【SYNTHETIC DEMO — not a customer】电商经营分析周报</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>周期: 2026-09-08 ~ 2026-09-14 (2026-W37周报) | 白牌交付: 代运营白牌数字化中心 | 勾稽质检: 100% PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>周期: 2026-09-08 ~ 2026-09-14 (Synthetic 2026-09-08 to 2026-09-14) | 白牌交付: 代运营白牌数字化中心 | 勾稽质检: True</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -593,7 +629,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>9.84%</t>
+          <t>9.84 %</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -613,7 +649,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>扣除退款后实际到账</t>
+          <t>订单额减退款，非到账</t>
         </is>
       </c>
     </row>
@@ -653,8 +689,10 @@
           <t>估算商品采购成本 (COGS)</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
-        <v>32621</v>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
@@ -665,11 +703,13 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>预估毛利润 (Gross Profit)</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>54734.97</v>
+          <t>预估广告后贡献利润 (Contribution after ads)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
@@ -680,17 +720,17 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>预估综合毛利率</t>
+          <t>预估综合广告后贡献利润率</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>50.04%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>毛利润 / 净销售额</t>
+          <t>广告后贡献利润 / 净销售额</t>
         </is>
       </c>
     </row>
@@ -724,47 +764,88 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
           <t>💡 高管经营洞察与运营建议:</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>【大盘概况】本周期全店实现 GMV ¥121,315.00，净销售额 ¥109,375.00，综合毛利率 50.0%，综合投产比 Blended ROI 为 5.51，经营处于健康盈利状态。</t>
+          <t>GMV ¥121,315.00；退款 ¥11,940.00；净销售额 ¥109,375.00。净销售额不代表到账。</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>【核心支柱】第一爆款【法式复古碎花连衣裙】贡献 GMV ¥33,813.00（占全店 27.9%），毛利贡献稳定。⚠️ 需紧急警惕库存仅剩 42 件，逼近断货线！</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>【止血建议】推广计划【引力魔方-新客拉新】持续亏损，花费 ¥6,528.35，投产比仅 0.95。建议立即压缩日预算 50% 以上，释放资金调优高产出计划。</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>【品质预警】单品【宽松廓形针织开衫】退款率高达 29.6%，造成 ¥2,847.00 营业额流失，需立即核查详情页版型参数及买家集中差评。</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>【下周聚焦】1) 追补第一爆款翻单；2) 砍除低效推广计划，预计下周可提升综合毛利率 3.5-5 个百分点；3) 将潜力爆款转为直通车核心测试组。</t>
+          <t>广告后贡献利润 N/A：成本、广告记录或退款退货成本规则不足；暂停利润结论。</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -791,8 +872,8 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -843,12 +924,12 @@
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>毛利润</t>
+          <t>广告后贡献利润</t>
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>毛利率</t>
+          <t>广告后贡献利润率</t>
         </is>
       </c>
     </row>
@@ -882,12 +963,14 @@
       <c r="I2" s="13" t="n">
         <v>6.31</v>
       </c>
-      <c r="J2" s="12" t="n">
-        <v>10218.36</v>
+      <c r="J2" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>53.8%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
     </row>
@@ -921,12 +1004,14 @@
       <c r="I3" s="13" t="n">
         <v>5.1</v>
       </c>
-      <c r="J3" s="12" t="n">
-        <v>7140.91</v>
+      <c r="J3" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="K3" s="11" t="inlineStr">
         <is>
-          <t>49.4%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
     </row>
@@ -960,12 +1045,14 @@
       <c r="I4" s="13" t="n">
         <v>6.39</v>
       </c>
-      <c r="J4" s="12" t="n">
-        <v>10339.67</v>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="K4" s="11" t="inlineStr">
         <is>
-          <t>53.5%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
     </row>
@@ -999,12 +1086,14 @@
       <c r="I5" s="13" t="n">
         <v>5.84</v>
       </c>
-      <c r="J5" s="12" t="n">
-        <v>7966.22</v>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>50.1%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
     </row>
@@ -1038,12 +1127,14 @@
       <c r="I6" s="13" t="n">
         <v>3.49</v>
       </c>
-      <c r="J6" s="12" t="n">
-        <v>2959.36</v>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>34.0%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
     </row>
@@ -1077,12 +1168,14 @@
       <c r="I7" s="13" t="n">
         <v>5.38</v>
       </c>
-      <c r="J7" s="12" t="n">
-        <v>6597.24</v>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>47.7%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
     </row>
@@ -1116,12 +1209,14 @@
       <c r="I8" s="13" t="n">
         <v>6.11</v>
       </c>
-      <c r="J8" s="12" t="n">
-        <v>9513.209999999999</v>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>52.5%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
     </row>
@@ -1149,10 +1244,10 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
     <col width="40" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -1209,12 +1304,12 @@
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>预估毛利</t>
+          <t>预估广告后贡献利润</t>
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>毛利率</t>
+          <t>广告后贡献利润率</t>
         </is>
       </c>
       <c r="M1" s="3" t="inlineStr">
@@ -1263,7 +1358,7 @@
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.7 %</t>
         </is>
       </c>
       <c r="I2" s="12" t="n">
@@ -1272,12 +1367,14 @@
       <c r="J2" s="13" t="n">
         <v>4.66</v>
       </c>
-      <c r="K2" s="12" t="n">
-        <v>16148.66</v>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>51.7%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
       <c r="M2" s="11" t="n">
@@ -1285,12 +1382,12 @@
       </c>
       <c r="N2" s="7" t="inlineStr">
         <is>
-          <t>现金金牛</t>
+          <t>数据不足，暂停利润结论</t>
         </is>
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>库存告急: 仅剩42件 (警戒线50)</t>
+          <t>库存告急: 仅剩42.0件 (警戒线50.0)</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1421,7 @@
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>8.0%</t>
+          <t>8.0 %</t>
         </is>
       </c>
       <c r="I3" s="12" t="n">
@@ -1333,12 +1430,14 @@
       <c r="J3" s="13" t="n">
         <v>2.42</v>
       </c>
-      <c r="K3" s="12" t="n">
-        <v>8457.440000000001</v>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L3" s="11" t="inlineStr">
         <is>
-          <t>49.8%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
       <c r="M3" s="11" t="n">
@@ -1346,7 +1445,7 @@
       </c>
       <c r="N3" s="7" t="inlineStr">
         <is>
-          <t>潜力爆品</t>
+          <t>数据不足，暂停利润结论</t>
         </is>
       </c>
       <c r="O3" s="14" t="inlineStr">
@@ -1385,21 +1484,25 @@
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>5.6%</t>
+          <t>5.6 %</t>
         </is>
       </c>
       <c r="I4" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>10013</v>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>65.5%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
       <c r="M4" s="11" t="n">
@@ -1407,7 +1510,7 @@
       </c>
       <c r="N4" s="7" t="inlineStr">
         <is>
-          <t>潜力爆品</t>
+          <t>数据不足，暂停利润结论</t>
         </is>
       </c>
       <c r="O4" s="14" t="inlineStr">
@@ -1446,7 +1549,7 @@
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>5.6%</t>
+          <t>5.6 %</t>
         </is>
       </c>
       <c r="I5" s="12" t="n">
@@ -1455,12 +1558,14 @@
       <c r="J5" s="13" t="n">
         <v>3.28</v>
       </c>
-      <c r="K5" s="12" t="n">
-        <v>5704.07</v>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L5" s="11" t="inlineStr">
         <is>
-          <t>42.1%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
       <c r="M5" s="11" t="n">
@@ -1468,7 +1573,7 @@
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>潜力爆品</t>
+          <t>数据不足，暂停利润结论</t>
         </is>
       </c>
       <c r="O5" s="14" t="inlineStr">
@@ -1507,21 +1612,25 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>4.0 %</t>
         </is>
       </c>
       <c r="I6" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>7416</v>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>70.4%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
       <c r="M6" s="11" t="n">
@@ -1529,7 +1638,7 @@
       </c>
       <c r="N6" s="7" t="inlineStr">
         <is>
-          <t>潜力爆品</t>
+          <t>数据不足，暂停利润结论</t>
         </is>
       </c>
       <c r="O6" s="14" t="inlineStr">
@@ -1568,21 +1677,25 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>22.2 %</t>
         </is>
       </c>
       <c r="I7" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="12" t="n">
-        <v>5376</v>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
-          <t>68.7%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
       <c r="M7" s="11" t="n">
@@ -1590,7 +1703,7 @@
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>退款隐患</t>
+          <t>数据不足，暂停利润结论</t>
         </is>
       </c>
       <c r="O7" s="14" t="inlineStr">
@@ -1629,21 +1742,25 @@
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>29.6%</t>
+          <t>29.6 %</t>
         </is>
       </c>
       <c r="I8" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="12" t="n">
-        <v>4774</v>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>70.3%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
       <c r="M8" s="11" t="n">
@@ -1651,7 +1768,7 @@
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>退款隐患</t>
+          <t>数据不足，暂停利润结论</t>
         </is>
       </c>
       <c r="O8" s="14" t="inlineStr">
@@ -1690,7 +1807,7 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>15.8%</t>
+          <t>15.8 %</t>
         </is>
       </c>
       <c r="I9" s="12" t="n">
@@ -1699,12 +1816,14 @@
       <c r="J9" s="13" t="n">
         <v>0.95</v>
       </c>
-      <c r="K9" s="12" t="n">
-        <v>-4304.35</v>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L9" s="11" t="inlineStr">
         <is>
-          <t>-142.3%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
       <c r="M9" s="11" t="n">
@@ -1712,7 +1831,7 @@
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>吸血亏损</t>
+          <t>数据不足，暂停利润结论</t>
         </is>
       </c>
       <c r="O9" s="14" t="inlineStr">
@@ -1751,21 +1870,25 @@
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>2.9%</t>
+          <t>2.9 %</t>
         </is>
       </c>
       <c r="I10" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>2074</v>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>77.2%</t>
+          <t>N/A（未提供或口径不足） %</t>
         </is>
       </c>
       <c r="M10" s="11" t="n">
@@ -1773,7 +1896,7 @@
       </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>平销防守</t>
+          <t>数据不足，暂停利润结论</t>
         </is>
       </c>
       <c r="O10" s="14" t="inlineStr">
@@ -1812,21 +1935,23 @@
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.0 %</t>
         </is>
       </c>
       <c r="I11" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="13" t="n">
-        <v>0</v>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="K11" s="12" t="n">
         <v>1139</v>
       </c>
       <c r="L11" s="11" t="inlineStr">
         <is>
-          <t>75.3%</t>
+          <t>75.3 %</t>
         </is>
       </c>
       <c r="M11" s="11" t="n">
@@ -1834,7 +1959,7 @@
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>平销防守</t>
+          <t>贡献利润非负</t>
         </is>
       </c>
       <c r="O11" s="14" t="inlineStr">
@@ -2163,7 +2288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2177,15 +2302,51 @@
           <t>会计级勾稽自检结果 (Audit Trail)</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>核验时间: 2026-09-17 22:07:34 | 结论: 全部通过 PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>核验时间: 2026-09-19 18:58:36 | 结论: 全部通过 PASS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -2267,24 +2428,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>{"total_ad_spend": 22019.03, "campaign_spend_sum": 22019.03, "diff": 0.0, "passed": true}</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>profit_equation</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>{"gross_profit": 54734.97, "expected_profit": 54734.97, "diff": 0.0, "passed": true}</t>
+          <t>{"passed": true}</t>
         </is>
       </c>
     </row>

</xml_diff>